<commit_message>
feat(ColorTiming): 完成 BattleHud GF.UI 迁移
接入 BattleHudForm 与 Presentation，绑定 Boss1/Boss2 场景上下文，更新预制体、UITable 及生成镜像、迁移器和 PlayMode 测试，移除旧桥接职责。
</commit_message>
<xml_diff>
--- a/GameData/DataTables/Core/UITable.xlsx
+++ b/GameData/DataTables/Core/UITable.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R122473dbc519451b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="2" r:id="Rffcfd9be826b42f4"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet3" sheetId="3" r:id="R9b3cdb8892a14d1f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Re9391634456c4ab1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="2" r:id="R275d074fb411455c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet3" sheetId="3" r:id="R7698ea822b124900"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -604,13 +604,27 @@
     </x:row>
     <x:row r="9">
       <x:c r="A9"/>
-      <x:c r="B9"/>
-      <x:c r="C9"/>
-      <x:c r="D9"/>
-      <x:c r="E9"/>
-      <x:c r="F9"/>
-      <x:c r="G9"/>
-      <x:c r="H9"/>
+      <x:c r="B9" t="n">
+        <x:v>1005</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>ColorTiming battle HUD</x:v>
+      </x:c>
+      <x:c r="D9" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="E9" t="str">
+        <x:v>ColorTiming/Game/BattleHud</x:v>
+      </x:c>
+      <x:c r="F9" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="G9" t="n">
+        <x:v>1</x:v>
+      </x:c>
+      <x:c r="H9" s="2" t="b">
+        <x:v>0</x:v>
+      </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
refactor(ColorTiming): 统一 UI 命名与迁移结构
统一 Loading、BattleHud、BattleResult、MainMenu、PauseMenu、HeroHP_Item 与 BossHP_Item 的节点命名，更新场景绑定、UI 表、迁移校验与规范证据；保留真实 PlayMode 验证状态。
</commit_message>
<xml_diff>
--- a/GameData/DataTables/Core/UITable.xlsx
+++ b/GameData/DataTables/Core/UITable.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Re9391634456c4ab1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="2" r:id="R275d074fb411455c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet3" sheetId="3" r:id="R7698ea822b124900"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R25b2885d357e4ee2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet2" sheetId="2" r:id="R0688f3509d00408a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet3" sheetId="3" r:id="R0ec619d69ee141eb"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -518,7 +518,7 @@
         <x:v>0</x:v>
       </x:c>
       <x:c r="E5" t="str">
-        <x:v>ColorTiming/Game/Esc</x:v>
+        <x:v>ColorTiming/Game/PauseMenu</x:v>
       </x:c>
       <x:c r="F5" s="2" t="b">
         <x:v>0</x:v>

</xml_diff>